<commit_message>
feat(wishbone): name Excel sheet tabs; share the broadcast window offset
Excel export: field sheets are now regfile_<sheet> and address-map sheets bus_map_<bus> (clamped to the 31-char sheet limit). The header row no longer sets a fixed height, so Excel auto-fits the wrapped 2-line header instead of clipping it; the Reset Value (Dec) column gets an explicit width so its label stays 2 lines.

wishbone-bus: each broadcast group now emits one shared <group>_off wire (adr - base) instead of repeating the subtraction in every subscriber address assign; the combo and pipe emit paths both reference it.

Tests, help and docs updated; soc/hbm demos regenerated.
</commit_message>
<xml_diff>
--- a/demo/hbm/fw/gen/wishbone/bus_regfiles.xlsx
+++ b/demo/hbm/fw/gen/wishbone/bus_regfiles.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="aword" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="center" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="dword" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="hbm" state="visible" r:id="rId7"/>
+    <sheet sheetId="1" name="regfile_aword" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="regfile_center" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="regfile_dword" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="bus_map_hbm" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -1243,10 +1243,10 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="10" max="12" width="16" customWidth="1"/>
+    <col min="9" max="12" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1869,10 +1869,10 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="10" max="12" width="16" customWidth="1"/>
+    <col min="9" max="12" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2343,10 +2343,10 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="10" max="12" width="16" customWidth="1"/>
+    <col min="9" max="12" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>